<commit_message>
Bulk Archived 12 ROs
</commit_message>
<xml_diff>
--- a/delivered_database.xlsx
+++ b/delivered_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M39"/>
+  <dimension ref="A1:M51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,10 +484,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>43739748</t>
-        </is>
+      <c r="A2" t="n">
+        <v>43739748</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -515,10 +513,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>43876954</t>
-        </is>
+      <c r="A3" t="n">
+        <v>43876954</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
@@ -546,10 +542,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>43731115</t>
-        </is>
+      <c r="A4" t="n">
+        <v>43731115</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
@@ -577,10 +571,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>43740749</t>
-        </is>
+      <c r="A5" t="n">
+        <v>43740749</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
@@ -608,10 +600,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>43766667</t>
-        </is>
+      <c r="A6" t="n">
+        <v>43766667</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
@@ -639,10 +629,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>43773523</t>
-        </is>
+      <c r="A7" t="n">
+        <v>43773523</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
@@ -670,10 +658,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>43845541</t>
-        </is>
+      <c r="A8" t="n">
+        <v>43845541</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
@@ -701,10 +687,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>43898787</t>
-        </is>
+      <c r="A9" t="n">
+        <v>43898787</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
@@ -732,10 +716,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>43657132</t>
-        </is>
+      <c r="A10" t="n">
+        <v>43657132</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
@@ -763,10 +745,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>43679913</t>
-        </is>
+      <c r="A11" t="n">
+        <v>43679913</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
@@ -794,10 +774,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>43769760</t>
-        </is>
+      <c r="A12" t="n">
+        <v>43769760</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
@@ -825,10 +803,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>43774711</t>
-        </is>
+      <c r="A13" t="n">
+        <v>43774711</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
@@ -856,10 +832,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>43859490</t>
-        </is>
+      <c r="A14" t="n">
+        <v>43859490</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
@@ -887,10 +861,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>43857037</t>
-        </is>
+      <c r="A15" t="n">
+        <v>43857037</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
@@ -918,10 +890,8 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>43895002</t>
-        </is>
+      <c r="A16" t="n">
+        <v>43895002</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
@@ -949,10 +919,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>43929831</t>
-        </is>
+      <c r="A17" t="n">
+        <v>43929831</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
@@ -980,10 +948,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>43862715</t>
-        </is>
+      <c r="A18" t="n">
+        <v>43862715</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
@@ -1011,10 +977,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>43718642</t>
-        </is>
+      <c r="A19" t="n">
+        <v>43718642</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
@@ -1046,10 +1010,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>43995897</t>
-        </is>
+      <c r="A20" t="n">
+        <v>43995897</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
@@ -1081,10 +1043,8 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>43725091</t>
-        </is>
+      <c r="A21" t="n">
+        <v>43725091</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
@@ -1116,10 +1076,8 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>43788065</t>
-        </is>
+      <c r="A22" t="n">
+        <v>43788065</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
@@ -1151,10 +1109,8 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>44015908</t>
-        </is>
+      <c r="A23" t="n">
+        <v>44015908</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
@@ -1186,10 +1142,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>44019770</t>
-        </is>
+      <c r="A24" t="n">
+        <v>44019770</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
@@ -1225,10 +1179,8 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>44005603</t>
-        </is>
+      <c r="A25" t="n">
+        <v>44005603</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
@@ -1276,10 +1228,8 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>44069146</t>
-        </is>
+      <c r="A26" t="n">
+        <v>44069146</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
@@ -1307,10 +1257,8 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>43997465</t>
-        </is>
+      <c r="A27" t="n">
+        <v>43997465</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
@@ -1342,10 +1290,8 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>43847772</t>
-        </is>
+      <c r="A28" t="n">
+        <v>43847772</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
@@ -1377,10 +1323,8 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>44020441</t>
-        </is>
+      <c r="A29" t="n">
+        <v>44020441</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
@@ -1408,10 +1352,8 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>44070325</t>
-        </is>
+      <c r="A30" t="n">
+        <v>44070325</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
@@ -1439,10 +1381,8 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>44076865</t>
-        </is>
+      <c r="A31" t="n">
+        <v>44076865</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
@@ -1498,10 +1438,8 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>44137008</t>
-        </is>
+      <c r="A32" t="n">
+        <v>44137008</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
@@ -1537,10 +1475,8 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>44139320</t>
-        </is>
+      <c r="A33" t="n">
+        <v>44139320</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
@@ -1568,10 +1504,8 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>43694084</t>
-        </is>
+      <c r="A34" t="n">
+        <v>43694084</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
@@ -1599,10 +1533,8 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>43890408</t>
-        </is>
+      <c r="A35" t="n">
+        <v>43890408</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
@@ -1638,10 +1570,8 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>44127301</t>
-        </is>
+      <c r="A36" t="n">
+        <v>44127301</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
@@ -1669,10 +1599,8 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>43942727</t>
-        </is>
+      <c r="A37" t="n">
+        <v>43942727</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1712,10 +1640,8 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>43653663</t>
-        </is>
+      <c r="A38" t="n">
+        <v>43653663</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1759,10 +1685,8 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>43797585</t>
-        </is>
+      <c r="A39" t="n">
+        <v>43797585</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -1801,6 +1725,458 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>43658486</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>19/9 - RBND - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den:   ,Pnt:   ,Fit:   - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>29/09/2026 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>43785924</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">19/9 - RBND - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den:   ,Pnt:   ,Fit:   - PI send </t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>29/09/2026 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>44023023</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>WIP - Painting</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>21/9 - WIP - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den: 20/9 - Painting</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>29/09/2026 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>43769098</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>22/9 - RBND - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den:   ,Pnt:   ,Fit: 22/9 - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>29/09/2026 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>44040772</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>IAP - Approval Pending</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>22/9 - IAP - In:   ,Int:   ,Sur: 22/9 ,Dis:   - Approval Pending</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>29/09/2026 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>44066357</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>WIP - Painting</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>23/9 - WIP - In:   ,Int:   ,Sur: 21/9 ,Dis: 22/9 ,App: 22/9 ,Den: 22/9 - Painting</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>29/09/2026 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>44091013</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ISP - Survey Pending</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>23/9 - ISP - In:   ,Int: 23/9 - Survey Pending</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>29/09/2026 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>43883974</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>24/9 - RBND - In: 3/9 ,Dis:   ,Den:   ,Pnt:   ,Fit:   - Vehicle Ready (cashwork)</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>29/09/2026 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>43998631</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>WIP - Dismantle</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>24/9 - WIP - In:   ,Int: 22/9 ,Sur: 22/9 - Dismantle</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>29/09/2026 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>44011687</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>24/9 - WIP - In: 2/9 ,Int: 2/9 ,Sur: 2/9 ,Dis:   ,App:   ,Den:   ,Pnt: 20/9 - Fitting</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>29/09/2026 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>43732625</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>24/9 - RBND - In: 2/9 ,Int: 2/9 ,Sur: 2/9 ,Dis:   ,App:   ,Den:   ,Pnt:   ,Fit:   - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>29/09/2026 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>44163447</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>WIP - Dismantle</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>24/9 - WIP - In:   ,Int:   ,Sur:   - Dismantle</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>29/09/2026 12:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Bulk Archived 17 ROs
</commit_message>
<xml_diff>
--- a/delivered_database.xlsx
+++ b/delivered_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M51"/>
+  <dimension ref="A1:S68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,6 +480,36 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>Delivered_At</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>M_Category</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Insurance_Company</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Approval_Type</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Supp_Approval_Date</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Final_Insp_Date</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>DO_Date</t>
         </is>
       </c>
     </row>
@@ -511,6 +541,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -540,6 +576,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -569,6 +611,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -598,6 +646,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -627,6 +681,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -656,6 +716,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -685,6 +751,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -714,6 +786,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -743,6 +821,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -772,6 +856,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -801,6 +891,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -830,6 +926,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -859,6 +961,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -888,6 +996,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -917,6 +1031,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -946,6 +1066,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -975,6 +1101,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1008,6 +1140,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1041,6 +1179,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1074,6 +1218,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1107,6 +1257,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1140,6 +1296,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1177,6 +1339,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1226,6 +1394,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1255,6 +1429,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1288,6 +1468,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1321,6 +1507,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1350,6 +1542,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1379,6 +1577,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1436,6 +1640,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1473,6 +1683,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1502,6 +1718,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1531,6 +1753,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1568,6 +1796,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1597,6 +1831,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1638,6 +1878,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1683,6 +1929,12 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1724,12 +1976,16 @@
           <t>26/09/2026 12:48</t>
         </is>
       </c>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>43658486</t>
-        </is>
+      <c r="A40" t="n">
+        <v>43658486</v>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
@@ -1755,12 +2011,16 @@
           <t>29/09/2026 12:30</t>
         </is>
       </c>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>43785924</t>
-        </is>
+      <c r="A41" t="n">
+        <v>43785924</v>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
@@ -1786,12 +2046,16 @@
           <t>29/09/2026 12:30</t>
         </is>
       </c>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>44023023</t>
-        </is>
+      <c r="A42" t="n">
+        <v>44023023</v>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
@@ -1821,12 +2085,16 @@
           <t>29/09/2026 12:30</t>
         </is>
       </c>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>43769098</t>
-        </is>
+      <c r="A43" t="n">
+        <v>43769098</v>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
@@ -1856,12 +2124,16 @@
           <t>29/09/2026 12:30</t>
         </is>
       </c>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr"/>
+      <c r="S43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>44040772</t>
-        </is>
+      <c r="A44" t="n">
+        <v>44040772</v>
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
@@ -1891,12 +2163,16 @@
           <t>29/09/2026 12:30</t>
         </is>
       </c>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>44066357</t>
-        </is>
+      <c r="A45" t="n">
+        <v>44066357</v>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
@@ -1938,12 +2214,16 @@
           <t>29/09/2026 12:30</t>
         </is>
       </c>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>44091013</t>
-        </is>
+      <c r="A46" t="n">
+        <v>44091013</v>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
@@ -1973,12 +2253,16 @@
           <t>29/09/2026 12:30</t>
         </is>
       </c>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>43883974</t>
-        </is>
+      <c r="A47" t="n">
+        <v>43883974</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -2008,12 +2292,16 @@
           <t>29/09/2026 12:30</t>
         </is>
       </c>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>43998631</t>
-        </is>
+      <c r="A48" t="n">
+        <v>43998631</v>
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
@@ -2051,12 +2339,16 @@
           <t>29/09/2026 12:30</t>
         </is>
       </c>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr"/>
+      <c r="S48" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>44011687</t>
-        </is>
+      <c r="A49" t="n">
+        <v>44011687</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -2098,12 +2390,16 @@
           <t>29/09/2026 12:30</t>
         </is>
       </c>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>43732625</t>
-        </is>
+      <c r="A50" t="n">
+        <v>43732625</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -2141,12 +2437,16 @@
           <t>29/09/2026 12:30</t>
         </is>
       </c>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>44163447</t>
-        </is>
+      <c r="A51" t="n">
+        <v>44163447</v>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
@@ -2176,6 +2476,925 @@
           <t>29/09/2026 12:30</t>
         </is>
       </c>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr"/>
+      <c r="S51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>43888271</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>22/9-RBND-In: ,Int:22/9,Sur:22/9,Dis:22/9,App:22/9,Den:22/9,Pnt:22/9,Fit:22/9-Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>06/10/2026 14:57</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>44048543</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>23/9 - WIP - In:   ,Int:   ,Sur:   ,Dis: 22/9 ,App:   ,Den: 22/9 ,Pnt: 22/9 - Fitting</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>06/10/2026 14:57</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>43902289</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>IAP - Approval Pending</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>24/9 - IAP - In: 16/9 ,Int: 16/9 ,Sur: 16/9 ,Dis:   - investigation</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>06/10/2026 14:57</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr"/>
+      <c r="S54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>43689237</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>PNA</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>24/9 - PNA</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>06/10/2026 14:57</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>44135014</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>24/9 - WIP - In: 21/9 ,Int: 21/9 ,Sur: 22/9 ,Dis: 23/9 ,App: 22/9 ,Den: 23/9 ,Pnt: 24/9 - Fitting</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>06/10/2026 14:57</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr"/>
+      <c r="S56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>44171471</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>WIP - Dismantle</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>24/9 - WIP - In:   ,Int:   ,Sur:   - Dismantle</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>06/10/2026 14:57</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>43739478</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>28/9-RBND-In:11/9,Int:11/9,Sur:12/9,Dis: ,App:14/9,Den:22/9,Pnt:28/9,Fit: -Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>06/10/2026 14:57</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr"/>
+      <c r="S58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>44108850</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>28/9-RBND-In: ,Int:22/9,Sur:22/9,Dis:23/9,App:23/9,Den:23/9,Pnt: ,Fit:28/9-Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>06/10/2026 14:57</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
+      <c r="R59" t="inlineStr"/>
+      <c r="S59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>43938356</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>28/9-RBND-In: ,Int: ,Sur: ,Dis: ,App:22/9,Den:27/9,Pnt:27/9,Fit:28/9-Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>06/10/2026 14:57</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr"/>
+      <c r="R60" t="inlineStr"/>
+      <c r="S60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>43931687</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>PNA</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>28/9 - PNA - Part not available</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>06/10/2026 14:57</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>44049849</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>28/9-RBND-In: ,Int: ,Sur:21/9,Dis: ,App:22/9,Den:24/9,Pnt:26/9,Fit:28/9-Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>06/10/2026 14:57</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>44050017</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>28/9 - WIP - In:   ,Int:   ,Sur: 21/9 ,Dis: 21/9 ,App: 21/9 ,Den: 22/9 ,Pnt: 27/9 - Fitting</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>06/10/2026 14:57</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr"/>
+      <c r="S63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>44050137</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>WIP - Painting</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>28/9 - WIP - In:   ,Int:   ,Sur: 21/9 ,Dis: 28/9 ,App: 24/9 ,Den: 28/9 - Painting</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>06/10/2026 14:57</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr"/>
+      <c r="S64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>44146209</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>PNA</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>28/9 - PNA - Part not available</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>06/10/2026 14:57</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="inlineStr"/>
+      <c r="S65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>44274626</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>WIP - Painting</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>29/9 - WIP - In: 28/9 ,Int: 28/9 ,Sur: 28/9 ,Dis: 29/9 ,App: 29/9 ,Den: 29/9 - Painting</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>06/10/2026 14:57</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
+      <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr"/>
+      <c r="R66" t="inlineStr"/>
+      <c r="S66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>43809445</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>29/9 - WIP - In: 1/6 ,Int: 1/6 ,Sur: 2/6 ,Dis:   ,App: 22/6 ,Den:   ,Pnt:   - Fitting</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>06/10/2026 14:57</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
+      <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr"/>
+      <c r="R67" t="inlineStr"/>
+      <c r="S67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>43810667</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>29/9 - WIP - In: 18/8 ,Int: 18/8 ,Sur: 21/8 ,Dis:   ,App: 25/8 ,Den:   ,Pnt:   - Fitting</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>06/10/2026 14:57</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr"/>
+      <c r="P68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr"/>
+      <c r="R68" t="inlineStr"/>
+      <c r="S68" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Bulk Archived 23 ROs
</commit_message>
<xml_diff>
--- a/delivered_database.xlsx
+++ b/delivered_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S68"/>
+  <dimension ref="A1:S91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2484,10 +2484,8 @@
       <c r="S51" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>43888271</t>
-        </is>
+      <c r="A52" t="n">
+        <v>43888271</v>
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
@@ -2549,10 +2547,8 @@
       <c r="S52" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>44048543</t>
-        </is>
+      <c r="A53" t="n">
+        <v>44048543</v>
       </c>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr"/>
@@ -2598,10 +2594,8 @@
       <c r="S53" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>43902289</t>
-        </is>
+      <c r="A54" t="n">
+        <v>43902289</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -2651,10 +2645,8 @@
       <c r="S54" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>43689237</t>
-        </is>
+      <c r="A55" t="n">
+        <v>43689237</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -2700,10 +2692,8 @@
       <c r="S55" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>44135014</t>
-        </is>
+      <c r="A56" t="n">
+        <v>44135014</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -2765,10 +2755,8 @@
       <c r="S56" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>44171471</t>
-        </is>
+      <c r="A57" t="n">
+        <v>44171471</v>
       </c>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr"/>
@@ -2806,10 +2794,8 @@
       <c r="S57" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>43739478</t>
-        </is>
+      <c r="A58" t="n">
+        <v>43739478</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -2867,10 +2853,8 @@
       <c r="S58" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>44108850</t>
-        </is>
+      <c r="A59" t="n">
+        <v>44108850</v>
       </c>
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
@@ -2928,10 +2912,8 @@
       <c r="S59" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>43938356</t>
-        </is>
+      <c r="A60" t="n">
+        <v>43938356</v>
       </c>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr"/>
@@ -2981,10 +2963,8 @@
       <c r="S60" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>43931687</t>
-        </is>
+      <c r="A61" t="n">
+        <v>43931687</v>
       </c>
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr"/>
@@ -3026,10 +3006,8 @@
       <c r="S61" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>44049849</t>
-        </is>
+      <c r="A62" t="n">
+        <v>44049849</v>
       </c>
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr"/>
@@ -3083,10 +3061,8 @@
       <c r="S62" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>44050017</t>
-        </is>
+      <c r="A63" t="n">
+        <v>44050017</v>
       </c>
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr"/>
@@ -3140,10 +3116,8 @@
       <c r="S63" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>44050137</t>
-        </is>
+      <c r="A64" t="n">
+        <v>44050137</v>
       </c>
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr"/>
@@ -3193,10 +3167,8 @@
       <c r="S64" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>44146209</t>
-        </is>
+      <c r="A65" t="n">
+        <v>44146209</v>
       </c>
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr"/>
@@ -3230,10 +3202,8 @@
       <c r="S65" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>44274626</t>
-        </is>
+      <c r="A66" t="n">
+        <v>44274626</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -3291,10 +3261,8 @@
       <c r="S66" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>43809445</t>
-        </is>
+      <c r="A67" t="n">
+        <v>43809445</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -3344,10 +3312,8 @@
       <c r="S67" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>43810667</t>
-        </is>
+      <c r="A68" t="n">
+        <v>43810667</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -3396,6 +3362,1181 @@
       <c r="R68" t="inlineStr"/>
       <c r="S68" t="inlineStr"/>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>44102135</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>22/9 - WIP - In:   ,Dis:   ,Den:   ,Pnt:   - Fitting (cashwork)</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr"/>
+      <c r="P69" t="inlineStr"/>
+      <c r="Q69" t="inlineStr"/>
+      <c r="R69" t="inlineStr"/>
+      <c r="S69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>44145099</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ISP - Claim Intimation Pending</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>23/9 - ISP - In:   - Claim Intimation Pending</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
+      <c r="P70" t="inlineStr"/>
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="inlineStr"/>
+      <c r="S70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>43739097</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>24/9 - WIP - In: 8/8 ,Int: 8/8 ,Sur: 11/8 ,Dis:   ,App: 11/8 ,Den:   ,Pnt:   - Fitting</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr"/>
+      <c r="P71" t="inlineStr"/>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="inlineStr"/>
+      <c r="S71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>43849704</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>IAP - Approval Pending</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>28/9 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - No Claim</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr"/>
+      <c r="P72" t="inlineStr"/>
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="inlineStr"/>
+      <c r="S72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>43857886</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>IAP - Approval Pending</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>29/9 - IAP - In: 14/9 ,Int: 21/9 ,Sur: 21/9 ,Dis:   - Investigation</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr"/>
+      <c r="P73" t="inlineStr"/>
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" t="inlineStr"/>
+      <c r="S73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>44044364</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>IAP - Approval Pending</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>29/9 - IAP - In: 19/9 ,Int: 20/9 ,Sur: 22/9 ,Dis:   - Approval Pending</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
+      <c r="P74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="inlineStr"/>
+      <c r="S74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>43739311</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>5/10-RBND-In:3/9,Int:3/9,Sur:3/9,Dis: ,App:9/9,Den:28/9,Pnt:29/9,Fit:4/10-Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr"/>
+      <c r="P75" t="inlineStr"/>
+      <c r="Q75" t="inlineStr"/>
+      <c r="R75" t="inlineStr"/>
+      <c r="S75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>44228604</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>5/10 - RBND - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den: 29/9 ,Pnt: 30/9 ,Fit: 5/10 - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr"/>
+      <c r="P76" t="inlineStr"/>
+      <c r="Q76" t="inlineStr"/>
+      <c r="R76" t="inlineStr"/>
+      <c r="S76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>44163189</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>WIP - Painting</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>5/10 - WIP - In:   ,Int:   ,Sur:   ,Dis: 5/10 ,App:   ,Den: 5/10 - Painting</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr"/>
+      <c r="O77" t="inlineStr"/>
+      <c r="P77" t="inlineStr"/>
+      <c r="Q77" t="inlineStr"/>
+      <c r="R77" t="inlineStr"/>
+      <c r="S77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>43809794</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>5/10 - WIP - In: 27/8 ,Int: 3/9 ,Sur: 4/9 ,Dis:   ,App: 7/9 ,Den:   ,Pnt:   - Fitting</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr"/>
+      <c r="P78" t="inlineStr"/>
+      <c r="Q78" t="inlineStr"/>
+      <c r="R78" t="inlineStr"/>
+      <c r="S78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>44089995</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr"/>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>WIP - Dismantle</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>5/10 - WIP - In:   ,Int:   ,Sur:   - Dismantle</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr"/>
+      <c r="O79" t="inlineStr"/>
+      <c r="P79" t="inlineStr"/>
+      <c r="Q79" t="inlineStr"/>
+      <c r="R79" t="inlineStr"/>
+      <c r="S79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>44416078</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>WIP - Dismantle</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>5/10 - WIP - In: 14/9 ,Int: 15/9 ,Sur: 17/9 - Dismantle</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr"/>
+      <c r="O80" t="inlineStr"/>
+      <c r="P80" t="inlineStr"/>
+      <c r="Q80" t="inlineStr"/>
+      <c r="R80" t="inlineStr"/>
+      <c r="S80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>44044061</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>5/10-RBND-In: ,Int: ,Sur:20/9,Dis: ,App:25/9,Den:29/9,Pnt:4/10,Fit:5/10-Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr"/>
+      <c r="O81" t="inlineStr"/>
+      <c r="P81" t="inlineStr"/>
+      <c r="Q81" t="inlineStr"/>
+      <c r="R81" t="inlineStr"/>
+      <c r="S81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>43794910</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>6/10 - RBND - In: 1/9 ,Int: 1/9 ,Sur: 1/9 ,Dis:   ,App:   ,Den:   ,Pnt:   ,Fit: 6/10 - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr"/>
+      <c r="O82" t="inlineStr"/>
+      <c r="P82" t="inlineStr"/>
+      <c r="Q82" t="inlineStr"/>
+      <c r="R82" t="inlineStr"/>
+      <c r="S82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>44437107</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr"/>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>6/10-RBND-In: ,Int:5/10,Sur:6/10,Dis:6/10,App:6/10,Den:6/10,Pnt:6/10,Fit:6/10-Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr"/>
+      <c r="O83" t="inlineStr"/>
+      <c r="P83" t="inlineStr"/>
+      <c r="Q83" t="inlineStr"/>
+      <c r="R83" t="inlineStr"/>
+      <c r="S83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>44438146</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr"/>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>WIP - Painting</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>6/10 - WIP - In:   ,Int: 5/10 ,Sur: 6/10 ,Dis: 6/10 ,App: 6/10 ,Den: 6/10 - Painting</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr"/>
+      <c r="O84" t="inlineStr"/>
+      <c r="P84" t="inlineStr"/>
+      <c r="Q84" t="inlineStr"/>
+      <c r="R84" t="inlineStr"/>
+      <c r="S84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>44485422</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr"/>
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>6/10 - WIP - In:   ,Dis: 6/10 ,Den: 6/10 ,Pnt: 6/10 - Fitting (cashwork)</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr"/>
+      <c r="O85" t="inlineStr"/>
+      <c r="P85" t="inlineStr"/>
+      <c r="Q85" t="inlineStr"/>
+      <c r="R85" t="inlineStr"/>
+      <c r="S85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>44437682</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr"/>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>6/10 - WIP - In:   ,Int: 5/10 ,Sur: 5/10 ,Dis: 6/10 ,App: 6/10 ,Den: 6/10 ,Pnt: 6/10 - Fitting</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr"/>
+      <c r="O86" t="inlineStr"/>
+      <c r="P86" t="inlineStr"/>
+      <c r="Q86" t="inlineStr"/>
+      <c r="R86" t="inlineStr"/>
+      <c r="S86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>44519271</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr"/>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>8/10 - WIP - In:   ,Int: 7/10 ,Sur: 7/10 ,Dis: 8/10 ,App: 8/10 ,Den: 8/10 ,Pnt: 8/10 - Fitting</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr"/>
+      <c r="O87" t="inlineStr"/>
+      <c r="P87" t="inlineStr"/>
+      <c r="Q87" t="inlineStr"/>
+      <c r="R87" t="inlineStr"/>
+      <c r="S87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>44526254</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr"/>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>8/10 - WIP - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den: 8/10 ,Pnt:   - Fitting</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr"/>
+      <c r="O88" t="inlineStr"/>
+      <c r="P88" t="inlineStr"/>
+      <c r="Q88" t="inlineStr"/>
+      <c r="R88" t="inlineStr"/>
+      <c r="S88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>WIP - Denting</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>9/10 - WIP - In: 1/10 ,Int: 2/10 ,Sur: 5/10 ,Dis: 8/10 ,App: 6/10 - Denting</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr"/>
+      <c r="O89" t="inlineStr"/>
+      <c r="P89" t="inlineStr"/>
+      <c r="Q89" t="inlineStr"/>
+      <c r="R89" t="inlineStr"/>
+      <c r="S89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>44004899</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>9/10-RBND-In:21/9,Int:21/9,Sur:21/9,Dis: ,App:22/9,Den: ,Pnt: ,Fit:8/10-Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr"/>
+      <c r="O90" t="inlineStr"/>
+      <c r="P90" t="inlineStr"/>
+      <c r="Q90" t="inlineStr"/>
+      <c r="R90" t="inlineStr"/>
+      <c r="S90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>44554153</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr"/>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>IAP - Approval Pending</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>9/10 - IAP - In:   ,Int: 8/10 ,Sur: 9/10 ,Dis:   - Approval Pending</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>10/10/2026 07:21</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr"/>
+      <c r="O91" t="inlineStr"/>
+      <c r="P91" t="inlineStr"/>
+      <c r="Q91" t="inlineStr"/>
+      <c r="R91" t="inlineStr"/>
+      <c r="S91" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Bulk Archived 29 ROs
</commit_message>
<xml_diff>
--- a/delivered_database.xlsx
+++ b/delivered_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S91"/>
+  <dimension ref="A1:S120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3363,10 +3363,8 @@
       <c r="S68" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>44102135</t>
-        </is>
+      <c r="A69" t="n">
+        <v>44102135</v>
       </c>
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr"/>
@@ -3400,10 +3398,8 @@
       <c r="S69" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>44145099</t>
-        </is>
+      <c r="A70" t="n">
+        <v>44145099</v>
       </c>
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr"/>
@@ -3437,10 +3433,8 @@
       <c r="S70" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>43739097</t>
-        </is>
+      <c r="A71" t="n">
+        <v>43739097</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -3490,10 +3484,8 @@
       <c r="S71" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>43849704</t>
-        </is>
+      <c r="A72" t="n">
+        <v>43849704</v>
       </c>
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr"/>
@@ -3527,10 +3519,8 @@
       <c r="S72" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>43857886</t>
-        </is>
+      <c r="A73" t="n">
+        <v>43857886</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -3580,10 +3570,8 @@
       <c r="S73" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>44044364</t>
-        </is>
+      <c r="A74" t="n">
+        <v>44044364</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -3629,10 +3617,8 @@
       <c r="S74" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>43739311</t>
-        </is>
+      <c r="A75" t="n">
+        <v>43739311</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -3694,10 +3680,8 @@
       <c r="S75" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>44228604</t>
-        </is>
+      <c r="A76" t="n">
+        <v>44228604</v>
       </c>
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr"/>
@@ -3743,10 +3727,8 @@
       <c r="S76" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>44163189</t>
-        </is>
+      <c r="A77" t="n">
+        <v>44163189</v>
       </c>
       <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr"/>
@@ -3788,10 +3770,8 @@
       <c r="S77" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>43809794</t>
-        </is>
+      <c r="A78" t="n">
+        <v>43809794</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -3841,10 +3821,8 @@
       <c r="S78" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>44089995</t>
-        </is>
+      <c r="A79" t="n">
+        <v>44089995</v>
       </c>
       <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr"/>
@@ -3882,10 +3860,8 @@
       <c r="S79" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>44416078</t>
-        </is>
+      <c r="A80" t="n">
+        <v>44416078</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -3935,10 +3911,8 @@
       <c r="S80" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>44044061</t>
-        </is>
+      <c r="A81" t="n">
+        <v>44044061</v>
       </c>
       <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr"/>
@@ -3992,10 +3966,8 @@
       <c r="S81" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>43794910</t>
-        </is>
+      <c r="A82" t="n">
+        <v>43794910</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -4045,10 +4017,8 @@
       <c r="S82" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>44437107</t>
-        </is>
+      <c r="A83" t="n">
+        <v>44437107</v>
       </c>
       <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr">
@@ -4110,10 +4080,8 @@
       <c r="S83" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>44438146</t>
-        </is>
+      <c r="A84" t="n">
+        <v>44438146</v>
       </c>
       <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr">
@@ -4167,10 +4135,8 @@
       <c r="S84" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>44485422</t>
-        </is>
+      <c r="A85" t="n">
+        <v>44485422</v>
       </c>
       <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr"/>
@@ -4216,10 +4182,8 @@
       <c r="S85" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>44437682</t>
-        </is>
+      <c r="A86" t="n">
+        <v>44437682</v>
       </c>
       <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr">
@@ -4277,10 +4241,8 @@
       <c r="S86" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>44519271</t>
-        </is>
+      <c r="A87" t="n">
+        <v>44519271</v>
       </c>
       <c r="B87" t="inlineStr"/>
       <c r="C87" t="inlineStr">
@@ -4338,10 +4300,8 @@
       <c r="S87" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>44526254</t>
-        </is>
+      <c r="A88" t="n">
+        <v>44526254</v>
       </c>
       <c r="B88" t="inlineStr"/>
       <c r="C88" t="inlineStr"/>
@@ -4379,10 +4339,8 @@
       <c r="S88" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>12345678</t>
-        </is>
+      <c r="A89" t="n">
+        <v>12345678</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -4436,10 +4394,8 @@
       <c r="S89" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>44004899</t>
-        </is>
+      <c r="A90" t="n">
+        <v>44004899</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -4493,10 +4449,8 @@
       <c r="S90" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>44554153</t>
-        </is>
+      <c r="A91" t="n">
+        <v>44554153</v>
       </c>
       <c r="B91" t="inlineStr"/>
       <c r="C91" t="inlineStr">
@@ -4537,6 +4491,1515 @@
       <c r="R91" t="inlineStr"/>
       <c r="S91" t="inlineStr"/>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>43681230</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr"/>
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>21/9 - RBND - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den:   ,Pnt:   ,Fit: 20/9 - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr"/>
+      <c r="O92" t="inlineStr"/>
+      <c r="P92" t="inlineStr"/>
+      <c r="Q92" t="inlineStr"/>
+      <c r="R92" t="inlineStr"/>
+      <c r="S92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>44173725</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr"/>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>IAP - Approval Pending</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>24/9 - IAP - In:   ,Int:   ,Sur: 24/9 ,Dis:   - Approval Pending</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr"/>
+      <c r="O93" t="inlineStr"/>
+      <c r="P93" t="inlineStr"/>
+      <c r="Q93" t="inlineStr"/>
+      <c r="R93" t="inlineStr"/>
+      <c r="S93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>44260904</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr"/>
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>IAP - Approval Pending</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">29/9 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - No Claim </t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr"/>
+      <c r="O94" t="inlineStr"/>
+      <c r="P94" t="inlineStr"/>
+      <c r="Q94" t="inlineStr"/>
+      <c r="R94" t="inlineStr"/>
+      <c r="S94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>43819129</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>30/9 - WIP - In: 2/9 ,Int: 2/9 ,Sur: 2/9 ,Dis:   ,App:   ,Den: 27/9 ,Pnt: 30/9 - Fitting</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr"/>
+      <c r="O95" t="inlineStr"/>
+      <c r="P95" t="inlineStr"/>
+      <c r="Q95" t="inlineStr"/>
+      <c r="R95" t="inlineStr"/>
+      <c r="S95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>43717479</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>5/10-RBND-In:6/8,Int:7/8,Sur:12/8,Dis:30/8,App:14/8,Den: ,Pnt:20/9,Fit:4/10-DO awaited</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr"/>
+      <c r="O96" t="inlineStr"/>
+      <c r="P96" t="inlineStr"/>
+      <c r="Q96" t="inlineStr"/>
+      <c r="R96" t="inlineStr"/>
+      <c r="S96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>44261809</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr"/>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>WIP - Dismantle</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>5/10 - WIP - In:   ,Int: 28/9 ,Sur: 29/9 - Dismantle</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr"/>
+      <c r="O97" t="inlineStr"/>
+      <c r="P97" t="inlineStr"/>
+      <c r="Q97" t="inlineStr"/>
+      <c r="R97" t="inlineStr"/>
+      <c r="S97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>44439791</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr"/>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>WIP - Denting</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>6/10 - WIP - In:   ,Int: 5/10 ,Sur: 5/10 ,Dis: 6/10 ,App: 5/10 - Denting</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr"/>
+      <c r="O98" t="inlineStr"/>
+      <c r="P98" t="inlineStr"/>
+      <c r="Q98" t="inlineStr"/>
+      <c r="R98" t="inlineStr"/>
+      <c r="S98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>44109383</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>8/10 - RBND - In: 22/9 ,Int:   ,Sur:   ,Dis:   ,App:   ,Den:   ,Pnt: 6/10 ,Fit: 8/10 - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr"/>
+      <c r="O99" t="inlineStr"/>
+      <c r="P99" t="inlineStr"/>
+      <c r="Q99" t="inlineStr"/>
+      <c r="R99" t="inlineStr"/>
+      <c r="S99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>44210428</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr"/>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>8/10 - WIP - In: 25/9 ,Int: 26/9 ,Sur: 27/9 ,Dis:   ,App: 4/10 ,Den: 7/10 ,Pnt: 8/10 - Fitting</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr"/>
+      <c r="O100" t="inlineStr"/>
+      <c r="P100" t="inlineStr"/>
+      <c r="Q100" t="inlineStr"/>
+      <c r="R100" t="inlineStr"/>
+      <c r="S100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>44524049</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr"/>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr"/>
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>IAP - Approval Pending</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>8/10 - IAP - In:   ,Int: 7/10 ,Sur: 7/10 ,Dis:   - Approval Pending</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr"/>
+      <c r="O101" t="inlineStr"/>
+      <c r="P101" t="inlineStr"/>
+      <c r="Q101" t="inlineStr"/>
+      <c r="R101" t="inlineStr"/>
+      <c r="S101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>44356089</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr"/>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>8/10-RBND-In: ,Int:5/10,Sur:5/10,Dis:8/10,App:8/10,Den:8/10,Pnt:8/10,Fit:8/10-Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr"/>
+      <c r="O102" t="inlineStr"/>
+      <c r="P102" t="inlineStr"/>
+      <c r="Q102" t="inlineStr"/>
+      <c r="R102" t="inlineStr"/>
+      <c r="S102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>44452638</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr"/>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>8/10-RBND-In: ,Int:5/10,Sur:5/10,Dis:5/10,App:5/10,Den:6/10,Pnt:6/10,Fit:8/10-Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr"/>
+      <c r="O103" t="inlineStr"/>
+      <c r="P103" t="inlineStr"/>
+      <c r="Q103" t="inlineStr"/>
+      <c r="R103" t="inlineStr"/>
+      <c r="S103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>43998801</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr"/>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>WIP - Painting</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>9/10 - WIP - In: 18/9 ,Int: 21/9 ,Sur: 21/9 ,Dis: 9/10 ,App: 30/9 ,Den: 9/10 - Painting</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr"/>
+      <c r="O104" t="inlineStr"/>
+      <c r="P104" t="inlineStr"/>
+      <c r="Q104" t="inlineStr"/>
+      <c r="R104" t="inlineStr"/>
+      <c r="S104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>44376284</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr"/>
+      <c r="C105" t="inlineStr"/>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr"/>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>9/10 - RBND - In:   ,Int:   ,Sur:   ,Dis:   ,App: 3/10 ,Den:   ,Pnt:   ,Fit: 9/10 - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr"/>
+      <c r="O105" t="inlineStr"/>
+      <c r="P105" t="inlineStr"/>
+      <c r="Q105" t="inlineStr"/>
+      <c r="R105" t="inlineStr"/>
+      <c r="S105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>44438700</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr"/>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>WIP - Denting</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>9/10 - WIP - In:   ,Int: 5/10 ,Sur: 8/10 ,Dis:   ,App: 9/10 - Denting</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr"/>
+      <c r="O106" t="inlineStr"/>
+      <c r="P106" t="inlineStr"/>
+      <c r="Q106" t="inlineStr"/>
+      <c r="R106" t="inlineStr"/>
+      <c r="S106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>44438589</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr"/>
+      <c r="C107" t="inlineStr"/>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>WIP - Denting</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>9/10 - WIP - In:   ,Int:   ,Sur: 8/10 ,Dis:   ,App: 9/10 - Denting</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N107" t="inlineStr"/>
+      <c r="O107" t="inlineStr"/>
+      <c r="P107" t="inlineStr"/>
+      <c r="Q107" t="inlineStr"/>
+      <c r="R107" t="inlineStr"/>
+      <c r="S107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>44439724</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr"/>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr"/>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>9/10-RBND-In: ,Int:5/10,Sur:5/10,Dis: ,App:5/10,Den:9/10,Pnt:9/10,Fit: -Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr"/>
+      <c r="O108" t="inlineStr"/>
+      <c r="P108" t="inlineStr"/>
+      <c r="Q108" t="inlineStr"/>
+      <c r="R108" t="inlineStr"/>
+      <c r="S108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>44533152</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr"/>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr"/>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>WIP - Painting</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>9/10 - WIP - In:   ,Int: 7/10 ,Sur: 8/10 ,Dis: 9/10 ,App: 9/10 ,Den: 9/10 - Painting</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr"/>
+      <c r="O109" t="inlineStr"/>
+      <c r="P109" t="inlineStr"/>
+      <c r="Q109" t="inlineStr"/>
+      <c r="R109" t="inlineStr"/>
+      <c r="S109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>44554776</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr"/>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr"/>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>9/10 - WIP - In:   ,Int: 8/10 ,Sur: 8/10 ,Dis:   ,App: 9/10 ,Den:   ,Pnt:   - Fitting</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr"/>
+      <c r="O110" t="inlineStr"/>
+      <c r="P110" t="inlineStr"/>
+      <c r="Q110" t="inlineStr"/>
+      <c r="R110" t="inlineStr"/>
+      <c r="S110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>44593943</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr"/>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>WIP - Dismantle</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>9/10 - WIP - In:   ,Int: 9/10 ,Sur: 9/10 - Dismantle</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr"/>
+      <c r="O111" t="inlineStr"/>
+      <c r="P111" t="inlineStr"/>
+      <c r="Q111" t="inlineStr"/>
+      <c r="R111" t="inlineStr"/>
+      <c r="S111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>44536059</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr"/>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>9/10 - WIP - In:   ,Int: 8/10 ,Sur: 8/10 ,Dis: 9/10 ,App: 8/10 ,Den: 9/10 ,Pnt:   - Fitting</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr"/>
+      <c r="O112" t="inlineStr"/>
+      <c r="P112" t="inlineStr"/>
+      <c r="Q112" t="inlineStr"/>
+      <c r="R112" t="inlineStr"/>
+      <c r="S112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>44566932</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr"/>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr"/>
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>IAP - Approval Pending</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>9/10 - IAP - In:   ,Int: 9/10 ,Sur: 9/10 ,Dis:   - Approval Pending</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N113" t="inlineStr"/>
+      <c r="O113" t="inlineStr"/>
+      <c r="P113" t="inlineStr"/>
+      <c r="Q113" t="inlineStr"/>
+      <c r="R113" t="inlineStr"/>
+      <c r="S113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>44567462</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr"/>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>WIP - Painting</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>9/10 - WIP - In:   ,Int: 8/10 ,Sur: 8/10 ,Dis: 9/10 ,App: 8/10 ,Den: 9/10 - Painting</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr"/>
+      <c r="O114" t="inlineStr"/>
+      <c r="P114" t="inlineStr"/>
+      <c r="Q114" t="inlineStr"/>
+      <c r="R114" t="inlineStr"/>
+      <c r="S114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>44567923</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr"/>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>IAP - Approval Pending</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>9/10 - IAP - In:   ,Int: 8/10 ,Sur: 8/10 ,Dis:   - Approval Pending</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N115" t="inlineStr"/>
+      <c r="O115" t="inlineStr"/>
+      <c r="P115" t="inlineStr"/>
+      <c r="Q115" t="inlineStr"/>
+      <c r="R115" t="inlineStr"/>
+      <c r="S115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>44592005</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr"/>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>9/10 - WIP - In:   ,Int: 8/10 ,Sur: 8/10 ,Dis: 9/10 ,App: 8/10 ,Den: 9/10 ,Pnt: 9/10 - Fitting</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N116" t="inlineStr"/>
+      <c r="O116" t="inlineStr"/>
+      <c r="P116" t="inlineStr"/>
+      <c r="Q116" t="inlineStr"/>
+      <c r="R116" t="inlineStr"/>
+      <c r="S116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>44614361</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr"/>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>WIP - Painting</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>10/10 - WIP - In:   ,Int: 7/10 ,Sur: 9/10 ,Dis: 10/10 ,App: 9/10 ,Den: 10/10 - Painting</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N117" t="inlineStr"/>
+      <c r="O117" t="inlineStr"/>
+      <c r="P117" t="inlineStr"/>
+      <c r="Q117" t="inlineStr"/>
+      <c r="R117" t="inlineStr"/>
+      <c r="S117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>44613813</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr"/>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr"/>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>ISP - Survey Pending</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>10/10 - ISP - In:   ,Int: 9/10 - Survey Pending</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N118" t="inlineStr"/>
+      <c r="O118" t="inlineStr"/>
+      <c r="P118" t="inlineStr"/>
+      <c r="Q118" t="inlineStr"/>
+      <c r="R118" t="inlineStr"/>
+      <c r="S118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>44650312</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr"/>
+      <c r="C119" t="inlineStr"/>
+      <c r="D119" t="inlineStr"/>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>14/10 - RBND - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den:   ,Pnt:   ,Fit:   - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N119" t="inlineStr"/>
+      <c r="O119" t="inlineStr"/>
+      <c r="P119" t="inlineStr"/>
+      <c r="Q119" t="inlineStr"/>
+      <c r="R119" t="inlineStr"/>
+      <c r="S119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>44614679</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr"/>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>15/10-RBND-In: ,Int:9/10,Sur:9/10,Dis:12/10,App:12/10,Den:13/10,Pnt:14/10,Fit:15/10-Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>15/10/2026 15:21</t>
+        </is>
+      </c>
+      <c r="N120" t="inlineStr"/>
+      <c r="O120" t="inlineStr"/>
+      <c r="P120" t="inlineStr"/>
+      <c r="Q120" t="inlineStr"/>
+      <c r="R120" t="inlineStr"/>
+      <c r="S120" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Bulk Archived 26 ROs
</commit_message>
<xml_diff>
--- a/delivered_database.xlsx
+++ b/delivered_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S120"/>
+  <dimension ref="A1:S146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4492,10 +4492,8 @@
       <c r="S91" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>43681230</t>
-        </is>
+      <c r="A92" t="n">
+        <v>43681230</v>
       </c>
       <c r="B92" t="inlineStr"/>
       <c r="C92" t="inlineStr"/>
@@ -4533,10 +4531,8 @@
       <c r="S92" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>44173725</t>
-        </is>
+      <c r="A93" t="n">
+        <v>44173725</v>
       </c>
       <c r="B93" t="inlineStr"/>
       <c r="C93" t="inlineStr"/>
@@ -4574,10 +4570,8 @@
       <c r="S93" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>44260904</t>
-        </is>
+      <c r="A94" t="n">
+        <v>44260904</v>
       </c>
       <c r="B94" t="inlineStr"/>
       <c r="C94" t="inlineStr"/>
@@ -4611,10 +4605,8 @@
       <c r="S94" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>43819129</t>
-        </is>
+      <c r="A95" t="n">
+        <v>43819129</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -4668,10 +4660,8 @@
       <c r="S95" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>43717479</t>
-        </is>
+      <c r="A96" t="n">
+        <v>43717479</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -4733,10 +4723,8 @@
       <c r="S96" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>44261809</t>
-        </is>
+      <c r="A97" t="n">
+        <v>44261809</v>
       </c>
       <c r="B97" t="inlineStr"/>
       <c r="C97" t="inlineStr">
@@ -4782,10 +4770,8 @@
       <c r="S97" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>44439791</t>
-        </is>
+      <c r="A98" t="n">
+        <v>44439791</v>
       </c>
       <c r="B98" t="inlineStr"/>
       <c r="C98" t="inlineStr">
@@ -4835,10 +4821,8 @@
       <c r="S98" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>44109383</t>
-        </is>
+      <c r="A99" t="n">
+        <v>44109383</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -4884,10 +4868,8 @@
       <c r="S99" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>44210428</t>
-        </is>
+      <c r="A100" t="n">
+        <v>44210428</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -4945,10 +4927,8 @@
       <c r="S100" t="inlineStr"/>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>44524049</t>
-        </is>
+      <c r="A101" t="n">
+        <v>44524049</v>
       </c>
       <c r="B101" t="inlineStr"/>
       <c r="C101" t="inlineStr">
@@ -4990,10 +4970,8 @@
       <c r="S101" t="inlineStr"/>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>44356089</t>
-        </is>
+      <c r="A102" t="n">
+        <v>44356089</v>
       </c>
       <c r="B102" t="inlineStr"/>
       <c r="C102" t="inlineStr">
@@ -5055,10 +5033,8 @@
       <c r="S102" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>44452638</t>
-        </is>
+      <c r="A103" t="n">
+        <v>44452638</v>
       </c>
       <c r="B103" t="inlineStr"/>
       <c r="C103" t="inlineStr">
@@ -5120,10 +5096,8 @@
       <c r="S103" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>43998801</t>
-        </is>
+      <c r="A104" t="n">
+        <v>43998801</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -5181,10 +5155,8 @@
       <c r="S104" t="inlineStr"/>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>44376284</t>
-        </is>
+      <c r="A105" t="n">
+        <v>44376284</v>
       </c>
       <c r="B105" t="inlineStr"/>
       <c r="C105" t="inlineStr"/>
@@ -5226,10 +5198,8 @@
       <c r="S105" t="inlineStr"/>
     </row>
     <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>44438700</t>
-        </is>
+      <c r="A106" t="n">
+        <v>44438700</v>
       </c>
       <c r="B106" t="inlineStr"/>
       <c r="C106" t="inlineStr">
@@ -5275,10 +5245,8 @@
       <c r="S106" t="inlineStr"/>
     </row>
     <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>44438589</t>
-        </is>
+      <c r="A107" t="n">
+        <v>44438589</v>
       </c>
       <c r="B107" t="inlineStr"/>
       <c r="C107" t="inlineStr"/>
@@ -5320,10 +5288,8 @@
       <c r="S107" t="inlineStr"/>
     </row>
     <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>44439724</t>
-        </is>
+      <c r="A108" t="n">
+        <v>44439724</v>
       </c>
       <c r="B108" t="inlineStr"/>
       <c r="C108" t="inlineStr">
@@ -5377,10 +5343,8 @@
       <c r="S108" t="inlineStr"/>
     </row>
     <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>44533152</t>
-        </is>
+      <c r="A109" t="n">
+        <v>44533152</v>
       </c>
       <c r="B109" t="inlineStr"/>
       <c r="C109" t="inlineStr">
@@ -5434,10 +5398,8 @@
       <c r="S109" t="inlineStr"/>
     </row>
     <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>44554776</t>
-        </is>
+      <c r="A110" t="n">
+        <v>44554776</v>
       </c>
       <c r="B110" t="inlineStr"/>
       <c r="C110" t="inlineStr">
@@ -5483,10 +5445,8 @@
       <c r="S110" t="inlineStr"/>
     </row>
     <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>44593943</t>
-        </is>
+      <c r="A111" t="n">
+        <v>44593943</v>
       </c>
       <c r="B111" t="inlineStr"/>
       <c r="C111" t="inlineStr">
@@ -5532,10 +5492,8 @@
       <c r="S111" t="inlineStr"/>
     </row>
     <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>44536059</t>
-        </is>
+      <c r="A112" t="n">
+        <v>44536059</v>
       </c>
       <c r="B112" t="inlineStr"/>
       <c r="C112" t="inlineStr">
@@ -5589,10 +5547,8 @@
       <c r="S112" t="inlineStr"/>
     </row>
     <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>44566932</t>
-        </is>
+      <c r="A113" t="n">
+        <v>44566932</v>
       </c>
       <c r="B113" t="inlineStr"/>
       <c r="C113" t="inlineStr">
@@ -5634,10 +5590,8 @@
       <c r="S113" t="inlineStr"/>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>44567462</t>
-        </is>
+      <c r="A114" t="n">
+        <v>44567462</v>
       </c>
       <c r="B114" t="inlineStr"/>
       <c r="C114" t="inlineStr">
@@ -5691,10 +5645,8 @@
       <c r="S114" t="inlineStr"/>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>44567923</t>
-        </is>
+      <c r="A115" t="n">
+        <v>44567923</v>
       </c>
       <c r="B115" t="inlineStr"/>
       <c r="C115" t="inlineStr">
@@ -5736,10 +5688,8 @@
       <c r="S115" t="inlineStr"/>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>44592005</t>
-        </is>
+      <c r="A116" t="n">
+        <v>44592005</v>
       </c>
       <c r="B116" t="inlineStr"/>
       <c r="C116" t="inlineStr">
@@ -5801,10 +5751,8 @@
       <c r="S116" t="inlineStr"/>
     </row>
     <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>44614361</t>
-        </is>
+      <c r="A117" t="n">
+        <v>44614361</v>
       </c>
       <c r="B117" t="inlineStr"/>
       <c r="C117" t="inlineStr">
@@ -5858,10 +5806,8 @@
       <c r="S117" t="inlineStr"/>
     </row>
     <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>44613813</t>
-        </is>
+      <c r="A118" t="n">
+        <v>44613813</v>
       </c>
       <c r="B118" t="inlineStr"/>
       <c r="C118" t="inlineStr">
@@ -5899,10 +5845,8 @@
       <c r="S118" t="inlineStr"/>
     </row>
     <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>44650312</t>
-        </is>
+      <c r="A119" t="n">
+        <v>44650312</v>
       </c>
       <c r="B119" t="inlineStr"/>
       <c r="C119" t="inlineStr"/>
@@ -5936,10 +5880,8 @@
       <c r="S119" t="inlineStr"/>
     </row>
     <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>44614679</t>
-        </is>
+      <c r="A120" t="n">
+        <v>44614679</v>
       </c>
       <c r="B120" t="inlineStr"/>
       <c r="C120" t="inlineStr">
@@ -6000,6 +5942,1376 @@
       <c r="R120" t="inlineStr"/>
       <c r="S120" t="inlineStr"/>
     </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>44004793</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr"/>
+      <c r="C121" t="inlineStr"/>
+      <c r="D121" t="inlineStr"/>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr"/>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>19/9 - RBND - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den:   ,Pnt:   ,Fit:   - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N121" t="inlineStr"/>
+      <c r="O121" t="inlineStr"/>
+      <c r="P121" t="inlineStr"/>
+      <c r="Q121" t="inlineStr"/>
+      <c r="R121" t="inlineStr"/>
+      <c r="S121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>43715952</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>8/10-RBND-In:18/8,Int:18/8,Sur:18/8,Dis:21/9,App:25/8,Den:21/9,Pnt:27/9,Fit:8/10-Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N122" t="inlineStr"/>
+      <c r="O122" t="inlineStr"/>
+      <c r="P122" t="inlineStr"/>
+      <c r="Q122" t="inlineStr"/>
+      <c r="R122" t="inlineStr"/>
+      <c r="S122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>43877087</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>8/10-RBND-In:16/9,Int:16/9,Sur:16/9,Dis:21/9,App:18/9,Den:4/10,Pnt:5/10,Fit:8/10-DO Awaited</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N123" t="inlineStr"/>
+      <c r="O123" t="inlineStr"/>
+      <c r="P123" t="inlineStr"/>
+      <c r="Q123" t="inlineStr"/>
+      <c r="R123" t="inlineStr"/>
+      <c r="S123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>44557261</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr"/>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>WIP - Painting</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>8/10 - WIP - In:   ,Int: 7/10 ,Sur: 7/10 ,Dis: 7/10 ,App: 7/10 ,Den: 7/10 - Painting</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr"/>
+      <c r="O124" t="inlineStr"/>
+      <c r="P124" t="inlineStr"/>
+      <c r="Q124" t="inlineStr"/>
+      <c r="R124" t="inlineStr"/>
+      <c r="S124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>44479958</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr"/>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>PNA</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>9/10 - PNA - Part not available</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N125" t="inlineStr"/>
+      <c r="O125" t="inlineStr"/>
+      <c r="P125" t="inlineStr"/>
+      <c r="Q125" t="inlineStr"/>
+      <c r="R125" t="inlineStr"/>
+      <c r="S125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>44598047</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr"/>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr"/>
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>IAP - Approval Pending</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>9/10 - IAP - In:   ,Int: 8/10 ,Sur: 9/10 ,Dis:   - Approval Pending</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N126" t="inlineStr"/>
+      <c r="O126" t="inlineStr"/>
+      <c r="P126" t="inlineStr"/>
+      <c r="Q126" t="inlineStr"/>
+      <c r="R126" t="inlineStr"/>
+      <c r="S126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>43721281</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr"/>
+      <c r="C127" t="inlineStr"/>
+      <c r="D127" t="inlineStr"/>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>14/10 - WIP - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den: 3/10 ,Pnt: 14/10 - Fitting</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N127" t="inlineStr"/>
+      <c r="O127" t="inlineStr"/>
+      <c r="P127" t="inlineStr"/>
+      <c r="Q127" t="inlineStr"/>
+      <c r="R127" t="inlineStr"/>
+      <c r="S127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>44260223</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr"/>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>14/10-RBND-In: ,Int:26/9,Sur:27/9,Dis:7/10,App:3/10,Den:7/10,Pnt:14/10,Fit: -Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr"/>
+      <c r="O128" t="inlineStr"/>
+      <c r="P128" t="inlineStr"/>
+      <c r="Q128" t="inlineStr"/>
+      <c r="R128" t="inlineStr"/>
+      <c r="S128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>44261876</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr"/>
+      <c r="C129" t="inlineStr"/>
+      <c r="D129" t="inlineStr"/>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>14/10 - WIP - In:   - wca (cashwork)</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N129" t="inlineStr"/>
+      <c r="O129" t="inlineStr"/>
+      <c r="P129" t="inlineStr"/>
+      <c r="Q129" t="inlineStr"/>
+      <c r="R129" t="inlineStr"/>
+      <c r="S129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>44525631</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr"/>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>14/10 - WIP - In:   ,Int: 7/10 ,Sur: 7/10 ,Dis: 8/10 ,App: 7/10 ,Den: 8/10 ,Pnt: 14/10 - Fitting</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N130" t="inlineStr"/>
+      <c r="O130" t="inlineStr"/>
+      <c r="P130" t="inlineStr"/>
+      <c r="Q130" t="inlineStr"/>
+      <c r="R130" t="inlineStr"/>
+      <c r="S130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>44533924</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr"/>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>14/10-RBND-In: ,Int:7/10,Sur:7/10,Dis:13/10,App:13/10,Den:13/10,Pnt:14/10,Fit:14/10-Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N131" t="inlineStr"/>
+      <c r="O131" t="inlineStr"/>
+      <c r="P131" t="inlineStr"/>
+      <c r="Q131" t="inlineStr"/>
+      <c r="R131" t="inlineStr"/>
+      <c r="S131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>44648222</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr"/>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>WIP - Painting</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>14/10 - WIP - In:   ,Int: 7/10 ,Sur: 7/10 ,Dis: 14/10 ,App: 14/10 ,Den: 14/10 - Painting</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N132" t="inlineStr"/>
+      <c r="O132" t="inlineStr"/>
+      <c r="P132" t="inlineStr"/>
+      <c r="Q132" t="inlineStr"/>
+      <c r="R132" t="inlineStr"/>
+      <c r="S132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>44613052</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr"/>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr"/>
+      <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr"/>
+      <c r="I133" t="inlineStr"/>
+      <c r="J133" t="inlineStr"/>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>PNA</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>14/10 - PNA - Part not available</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N133" t="inlineStr"/>
+      <c r="O133" t="inlineStr"/>
+      <c r="P133" t="inlineStr"/>
+      <c r="Q133" t="inlineStr"/>
+      <c r="R133" t="inlineStr"/>
+      <c r="S133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>44145099</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr"/>
+      <c r="C134" t="inlineStr"/>
+      <c r="D134" t="inlineStr"/>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr"/>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>ISP - Claim Intimation Pending</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>14/10 - ISP - In:   - wca - No claim</t>
+        </is>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr"/>
+      <c r="O134" t="inlineStr"/>
+      <c r="P134" t="inlineStr"/>
+      <c r="Q134" t="inlineStr"/>
+      <c r="R134" t="inlineStr"/>
+      <c r="S134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>44762714</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr"/>
+      <c r="C135" t="inlineStr"/>
+      <c r="D135" t="inlineStr"/>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr"/>
+      <c r="G135" t="inlineStr"/>
+      <c r="H135" t="inlineStr"/>
+      <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr"/>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>PNA</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>15/10 - PNA - Part not available</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N135" t="inlineStr"/>
+      <c r="O135" t="inlineStr"/>
+      <c r="P135" t="inlineStr"/>
+      <c r="Q135" t="inlineStr"/>
+      <c r="R135" t="inlineStr"/>
+      <c r="S135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>44648547</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr"/>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>15/10-RBND-In:11/10,Int:12/10,Sur:14/10,Dis:15/10,App:15/10,Den:15/10,Pnt:15/10,Fit:15/10-VehicleRea</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N136" t="inlineStr"/>
+      <c r="O136" t="inlineStr"/>
+      <c r="P136" t="inlineStr"/>
+      <c r="Q136" t="inlineStr"/>
+      <c r="R136" t="inlineStr"/>
+      <c r="S136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>44725346</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr"/>
+      <c r="C137" t="inlineStr"/>
+      <c r="D137" t="inlineStr"/>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr"/>
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>15/10 - WIP - In:   ,Dis:   ,Den:   ,Pnt:   - Fitting (cashwork)</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N137" t="inlineStr"/>
+      <c r="O137" t="inlineStr"/>
+      <c r="P137" t="inlineStr"/>
+      <c r="Q137" t="inlineStr"/>
+      <c r="R137" t="inlineStr"/>
+      <c r="S137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>44455086</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr"/>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>15/10-RBND-In: ,Int:5/10,Sur:5/10,Dis:8/10,App:6/10,Den:13/10,Pnt:14/10,Fit:15/10-Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr"/>
+      <c r="O138" t="inlineStr"/>
+      <c r="P138" t="inlineStr"/>
+      <c r="Q138" t="inlineStr"/>
+      <c r="R138" t="inlineStr"/>
+      <c r="S138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>44627567</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr"/>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr"/>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>WIP - Fitting</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>16/10-WIP-In: ,Int:12/10,Sur:13/10,Dis:15/10,App:13/10,Den:16/10,Pnt:16/10-Fitting</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr"/>
+      <c r="O139" t="inlineStr"/>
+      <c r="P139" t="inlineStr"/>
+      <c r="Q139" t="inlineStr"/>
+      <c r="R139" t="inlineStr"/>
+      <c r="S139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>44790400</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr"/>
+      <c r="D140" t="inlineStr"/>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr"/>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>16/10 - WIP - In: 16/10 ,Dis: 16/10 ,Den: 16/10 ,Pnt: 16/10 - Fitting (cashwork)</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr"/>
+      <c r="O140" t="inlineStr"/>
+      <c r="P140" t="inlineStr"/>
+      <c r="Q140" t="inlineStr"/>
+      <c r="R140" t="inlineStr"/>
+      <c r="S140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>44366447</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr"/>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr"/>
+      <c r="I141" t="inlineStr"/>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>IAP - Approval Pending</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>16/10 - IAP - In:   ,Int: 5/10 ,Sur: 4/10 ,Dis: 15/10 - Approval pending Ticket - CAS-96544-S5W5G9</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr"/>
+      <c r="O141" t="inlineStr"/>
+      <c r="P141" t="inlineStr"/>
+      <c r="Q141" t="inlineStr"/>
+      <c r="R141" t="inlineStr"/>
+      <c r="S141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>44763240</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr"/>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr"/>
+      <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr"/>
+      <c r="I142" t="inlineStr"/>
+      <c r="J142" t="inlineStr"/>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>WIP - Denting</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>16/10 - WIP - In:   ,Int: 15/10 ,Sur: 14/10 ,Dis:   ,App: 15/10 - Denting</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr"/>
+      <c r="O142" t="inlineStr"/>
+      <c r="P142" t="inlineStr"/>
+      <c r="Q142" t="inlineStr"/>
+      <c r="R142" t="inlineStr"/>
+      <c r="S142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>44445280</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr"/>
+      <c r="J143" t="inlineStr"/>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>RBND - Vehicle Ready</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>16/10-RBND-In:5/10,Int:5/10,Sur:6/10,Dis:16/10,App:6/10,Den:16/10,Pnt:16/10,Fit: -PI Send</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr"/>
+      <c r="O143" t="inlineStr"/>
+      <c r="P143" t="inlineStr"/>
+      <c r="Q143" t="inlineStr"/>
+      <c r="R143" t="inlineStr"/>
+      <c r="S143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>44790920</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr"/>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr"/>
+      <c r="G144" t="inlineStr"/>
+      <c r="H144" t="inlineStr"/>
+      <c r="I144" t="inlineStr"/>
+      <c r="J144" t="inlineStr"/>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>IAP - Approval Pending</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>16/10 - IAP - In:   ,Int: 15/10 ,Sur: 16/10 ,Dis:   - Approval Pending</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N144" t="inlineStr"/>
+      <c r="O144" t="inlineStr"/>
+      <c r="P144" t="inlineStr"/>
+      <c r="Q144" t="inlineStr"/>
+      <c r="R144" t="inlineStr"/>
+      <c r="S144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>44798704</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr"/>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr"/>
+      <c r="I145" t="inlineStr"/>
+      <c r="J145" t="inlineStr"/>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>IAP - Approval Pending</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>16/10 - IAP - In:   ,Int: 15/10 ,Sur: 16/10 ,Dis:   - Approval Pending</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N145" t="inlineStr"/>
+      <c r="O145" t="inlineStr"/>
+      <c r="P145" t="inlineStr"/>
+      <c r="Q145" t="inlineStr"/>
+      <c r="R145" t="inlineStr"/>
+      <c r="S145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>44851902</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr"/>
+      <c r="C146" t="inlineStr"/>
+      <c r="D146" t="inlineStr"/>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr"/>
+      <c r="I146" t="inlineStr"/>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>19/10 - WIP - In:   ,Dis: 19/10 ,Den: 19/10 - Painting (cashwork)</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>21/10/2026 12:43</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr"/>
+      <c r="O146" t="inlineStr"/>
+      <c r="P146" t="inlineStr"/>
+      <c r="Q146" t="inlineStr"/>
+      <c r="R146" t="inlineStr"/>
+      <c r="S146" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>